<commit_message>
Refresh Shiny app data 2026-10-06 11:46
</commit_message>
<xml_diff>
--- a/Evo-M1 primary-data candidates (Sep 2026).xlsx
+++ b/Evo-M1 primary-data candidates (Sep 2026).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://alleninstitute.sharepoint.com/sites/MammalianM1/Shared Documents/General/Species/Evo-M1-Trait-Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1105" documentId="11_C2338D8A795ED50E97E819E7E0BCBE8359B1E8BC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{57C5DED8-C7E6-DD47-846D-F0F65A9AD149}"/>
+  <xr:revisionPtr revIDLastSave="1109" documentId="11_C2338D8A795ED50E97E819E7E0BCBE8359B1E8BC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{584A46E9-07A5-E441-ACBA-F4F76982F0C5}"/>
   <bookViews>
-    <workbookView xWindow="48840" yWindow="2800" windowWidth="21860" windowHeight="19540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20420" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
     <sheet name="Sequenced species" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="191028" refMode="R1C1" iterateCount="0" calcCompleted="0" calcOnSave="0" concurrentCalc="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -2640,11 +2640,11 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -2739,6 +2739,64 @@
           <bgColor rgb="FFFFD966"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+      </font>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+      </font>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+      </font>
+      <alignment vertical="top" wrapText="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+      </font>
+      <alignment vertical="top" wrapText="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+      </font>
+      <alignment vertical="top" wrapText="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+      </font>
+      <alignment vertical="top" wrapText="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <i/>
+        <name val="Calibri"/>
+      </font>
+      <alignment vertical="top" wrapText="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+      </font>
+      <alignment vertical="top" wrapText="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <name val="Calibri"/>
+      </font>
+      <alignment vertical="center"/>
     </dxf>
     <dxf>
       <font>
@@ -2896,64 +2954,6 @@
         <name val="Calibri"/>
       </font>
       <alignment vertical="center" wrapText="1"/>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Calibri"/>
-      </font>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Calibri"/>
-      </font>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Calibri"/>
-      </font>
-      <alignment vertical="top" wrapText="1"/>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Calibri"/>
-      </font>
-      <alignment vertical="top" wrapText="1"/>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Calibri"/>
-      </font>
-      <alignment vertical="top" wrapText="1"/>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Calibri"/>
-      </font>
-      <alignment vertical="top" wrapText="1"/>
-    </dxf>
-    <dxf>
-      <font>
-        <i/>
-        <name val="Calibri"/>
-      </font>
-      <alignment vertical="top" wrapText="1"/>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Calibri"/>
-      </font>
-      <alignment vertical="top" wrapText="1"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <name val="Calibri"/>
-      </font>
-      <alignment vertical="center"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -4204,50 +4204,43 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B265261E-B317-416F-8AB3-6E065E893377}" name="tblCandidates" displayName="tblCandidates" ref="A2:Q71" totalsRowShown="0" headerRowDxfId="26" dataDxfId="25">
-  <autoFilter ref="A2:Q71" xr:uid="{B265261E-B317-416F-8AB3-6E065E893377}">
-    <filterColumn colId="1">
-      <filters>
-        <filter val="P2"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B265261E-B317-416F-8AB3-6E065E893377}" name="tblCandidates" displayName="tblCandidates" ref="A2:Q71" totalsRowShown="0" headerRowDxfId="35" dataDxfId="34">
   <tableColumns count="17">
-    <tableColumn id="1" xr3:uid="{FB0B923B-BB8F-4FEF-849E-57604257D14F}" name="ID" dataDxfId="24"/>
-    <tableColumn id="2" xr3:uid="{9848EDB8-9369-4C0D-865C-D7666441960F}" name="Priority" dataDxfId="23"/>
-    <tableColumn id="3" xr3:uid="{240D3C05-212D-48EC-9089-312FB24B25B7}" name="Theme" dataDxfId="22"/>
-    <tableColumn id="4" xr3:uid="{802A2A12-2F09-4601-9439-90696431BA8F}" name="Region" dataDxfId="21"/>
-    <tableColumn id="5" xr3:uid="{3C2B75D3-7E75-46FF-8D3A-2E6373521950}" name="Citation" dataDxfId="20"/>
-    <tableColumn id="6" xr3:uid="{792400AE-D8B4-4430-AC52-17AB02C3074E}" name="DOI / identifier" dataDxfId="19"/>
-    <tableColumn id="7" xr3:uid="{AA2008FC-198F-40E0-8E00-E18B702092CA}" name="Link" dataDxfId="18" dataCellStyle="Hyperlink"/>
-    <tableColumn id="8" xr3:uid="{4375BD5D-A43C-4B68-998A-98E34A2F6BC2}" name="Primary data" dataDxfId="17"/>
-    <tableColumn id="9" xr3:uid="{A4502408-465D-47F1-846C-57609F384562}" name="Taxa / sample" dataDxfId="16"/>
-    <tableColumn id="10" xr3:uid="{B0050F33-9FCA-4DB4-9C9B-5D1D7E9D2F95}" name="Sequenced-species overlap" dataDxfId="15"/>
-    <tableColumn id="11" xr3:uid="{6E78D2B3-0467-4FD0-AC44-FD8716DADB8B}" name="Suggested home in repo" dataDxfId="14"/>
-    <tableColumn id="12" xr3:uid="{7EC3809C-6B6F-4E64-9F81-2EACB8108446}" name="Gap it fills" dataDxfId="13"/>
-    <tableColumn id="13" xr3:uid="{3BEF5209-EDBC-49DA-961B-1EB297249044}" name="Check before building" dataDxfId="12"/>
-    <tableColumn id="14" xr3:uid="{A518122D-0531-4D76-BBA7-ABFCC0F9B902}" name="Access" dataDxfId="11"/>
-    <tableColumn id="17" xr3:uid="{65D2F790-D948-4D92-8A38-C2A0B6E3BED1}" name="Holdings check" dataDxfId="10"/>
-    <tableColumn id="16" xr3:uid="{B663890F-DF3E-4D0C-A47F-5E0CCE8113FC}" name="Where it already appears" dataDxfId="9"/>
-    <tableColumn id="15" xr3:uid="{B1C64E1F-6D3C-468C-A7ED-F8122D3D319C}" name="Registry / roadmap status" dataDxfId="8"/>
+    <tableColumn id="1" xr3:uid="{FB0B923B-BB8F-4FEF-849E-57604257D14F}" name="ID" dataDxfId="33"/>
+    <tableColumn id="2" xr3:uid="{9848EDB8-9369-4C0D-865C-D7666441960F}" name="Priority" dataDxfId="32"/>
+    <tableColumn id="3" xr3:uid="{240D3C05-212D-48EC-9089-312FB24B25B7}" name="Theme" dataDxfId="31"/>
+    <tableColumn id="4" xr3:uid="{802A2A12-2F09-4601-9439-90696431BA8F}" name="Region" dataDxfId="30"/>
+    <tableColumn id="5" xr3:uid="{3C2B75D3-7E75-46FF-8D3A-2E6373521950}" name="Citation" dataDxfId="29"/>
+    <tableColumn id="6" xr3:uid="{792400AE-D8B4-4430-AC52-17AB02C3074E}" name="DOI / identifier" dataDxfId="28"/>
+    <tableColumn id="7" xr3:uid="{AA2008FC-198F-40E0-8E00-E18B702092CA}" name="Link" dataDxfId="27" dataCellStyle="Hyperlink"/>
+    <tableColumn id="8" xr3:uid="{4375BD5D-A43C-4B68-998A-98E34A2F6BC2}" name="Primary data" dataDxfId="26"/>
+    <tableColumn id="9" xr3:uid="{A4502408-465D-47F1-846C-57609F384562}" name="Taxa / sample" dataDxfId="25"/>
+    <tableColumn id="10" xr3:uid="{B0050F33-9FCA-4DB4-9C9B-5D1D7E9D2F95}" name="Sequenced-species overlap" dataDxfId="24"/>
+    <tableColumn id="11" xr3:uid="{6E78D2B3-0467-4FD0-AC44-FD8716DADB8B}" name="Suggested home in repo" dataDxfId="23"/>
+    <tableColumn id="12" xr3:uid="{7EC3809C-6B6F-4E64-9F81-2EACB8108446}" name="Gap it fills" dataDxfId="22"/>
+    <tableColumn id="13" xr3:uid="{3BEF5209-EDBC-49DA-961B-1EB297249044}" name="Check before building" dataDxfId="21"/>
+    <tableColumn id="14" xr3:uid="{A518122D-0531-4D76-BBA7-ABFCC0F9B902}" name="Access" dataDxfId="20"/>
+    <tableColumn id="17" xr3:uid="{65D2F790-D948-4D92-8A38-C2A0B6E3BED1}" name="Holdings check" dataDxfId="19"/>
+    <tableColumn id="16" xr3:uid="{B663890F-DF3E-4D0C-A47F-5E0CCE8113FC}" name="Where it already appears" dataDxfId="18"/>
+    <tableColumn id="15" xr3:uid="{B1C64E1F-6D3C-468C-A7ED-F8122D3D319C}" name="Registry / roadmap status" dataDxfId="17"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{02D14B67-E43C-4F79-A409-F681083E3122}" name="tblSpecies" displayName="tblSpecies" ref="A2:G27" totalsRowShown="0" headerRowDxfId="35" dataDxfId="34">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{02D14B67-E43C-4F79-A409-F681083E3122}" name="tblSpecies" displayName="tblSpecies" ref="A2:G27" totalsRowShown="0" headerRowDxfId="16" dataDxfId="15">
   <autoFilter ref="A2:G27" xr:uid="{02D14B67-E43C-4F79-A409-F681083E3122}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{7B3EE8BA-DF55-4C8B-9D9E-9104E407C941}" name="Species" dataDxfId="33"/>
-    <tableColumn id="2" xr3:uid="{00258CF3-23F2-4BBE-9F89-2BB5086708AB}" name="Common name" dataDxfId="32"/>
-    <tableColumn id="3" xr3:uid="{CAF2E8EA-0691-4013-8D71-9455B955AB6B}" name="Order" dataDxfId="31"/>
-    <tableColumn id="4" xr3:uid="{FF3272E7-41C7-4662-858F-3512F91CD347}" name="Confirmed in candidates" dataDxfId="30"/>
-    <tableColumn id="5" xr3:uid="{DFC7ABA0-8EF7-4B55-A0C3-7EF96FD83291}" name="Genus-level or unconfirmed" dataDxfId="29"/>
-    <tableColumn id="6" xr3:uid="{D0D09B95-BCA7-493B-92CD-222AB61DBC85}" name="Confirmed (n)" dataDxfId="28">
+    <tableColumn id="1" xr3:uid="{7B3EE8BA-DF55-4C8B-9D9E-9104E407C941}" name="Species" dataDxfId="14"/>
+    <tableColumn id="2" xr3:uid="{00258CF3-23F2-4BBE-9F89-2BB5086708AB}" name="Common name" dataDxfId="13"/>
+    <tableColumn id="3" xr3:uid="{CAF2E8EA-0691-4013-8D71-9455B955AB6B}" name="Order" dataDxfId="12"/>
+    <tableColumn id="4" xr3:uid="{FF3272E7-41C7-4662-858F-3512F91CD347}" name="Confirmed in candidates" dataDxfId="11"/>
+    <tableColumn id="5" xr3:uid="{DFC7ABA0-8EF7-4B55-A0C3-7EF96FD83291}" name="Genus-level or unconfirmed" dataDxfId="10"/>
+    <tableColumn id="6" xr3:uid="{D0D09B95-BCA7-493B-92CD-222AB61DBC85}" name="Confirmed (n)" dataDxfId="9">
       <calculatedColumnFormula>IF(TRIM(D3)="",0,LEN(D3)-LEN(SUBSTITUTE(D3,",",""))+1)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{8E94C980-5842-4D14-8184-A095ED353FF0}" name="Genus-level (n)" dataDxfId="27">
+    <tableColumn id="7" xr3:uid="{8E94C980-5842-4D14-8184-A095ED353FF0}" name="Genus-level (n)" dataDxfId="8">
       <calculatedColumnFormula>IF(TRIM(E3)="",0,LEN(E3)-LEN(SUBSTITUTE(E3,",",""))+1)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4554,11 +4547,11 @@
       <c r="B1" s="28"/>
     </row>
     <row r="2" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="30" t="str">
+      <c r="A2" s="29" t="str">
         <f>"Scouted September 2026 for Alexandra de Sousa · "&amp;ROWS(tblCandidates[ID])&amp;" candidates, "&amp;COUNTIF(tblCandidates[Priority],1)&amp;" at priority 1"</f>
         <v>Scouted September 2026 for Alexandra de Sousa · 69 candidates, 23 at priority 1</v>
       </c>
-      <c r="B2" s="30"/>
+      <c r="B2" s="29"/>
     </row>
     <row r="3" spans="1:2" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="15" t="s">
@@ -4787,7 +4780,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="3" spans="1:17" ht="44.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:17" ht="44.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>48</v>
       </c>
@@ -4895,7 +4888,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="5" spans="1:17" ht="44.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:17" ht="44.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="6" t="s">
         <v>73</v>
       </c>
@@ -4949,7 +4942,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="6" spans="1:17" ht="44.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:17" ht="44.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="6" t="s">
         <v>83</v>
       </c>
@@ -5003,7 +4996,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="7" spans="1:17" ht="57.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:17" ht="57.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="6" t="s">
         <v>93</v>
       </c>
@@ -5057,7 +5050,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="8" spans="1:17" ht="57.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:17" ht="57.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="6" t="s">
         <v>104</v>
       </c>
@@ -5111,7 +5104,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="9" spans="1:17" ht="57.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:17" ht="57.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="6" t="s">
         <v>115</v>
       </c>
@@ -5165,7 +5158,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="10" spans="1:17" ht="44.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:17" ht="44.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="6" t="s">
         <v>128</v>
       </c>
@@ -5219,7 +5212,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="11" spans="1:17" ht="71.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:17" ht="71.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="6" t="s">
         <v>138</v>
       </c>
@@ -5327,7 +5320,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="13" spans="1:17" ht="71.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:17" ht="71.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="6" t="s">
         <v>160</v>
       </c>
@@ -5435,7 +5428,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="15" spans="1:17" ht="71.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:17" ht="71.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="6" t="s">
         <v>180</v>
       </c>
@@ -5543,7 +5536,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="17" spans="1:17" ht="57.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:17" ht="57.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="6" t="s">
         <v>199</v>
       </c>
@@ -5597,7 +5590,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="18" spans="1:17" ht="57.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:17" ht="57.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="6" t="s">
         <v>209</v>
       </c>
@@ -5651,7 +5644,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="19" spans="1:17" ht="57.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:17" ht="57.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="6" t="s">
         <v>217</v>
       </c>
@@ -5867,7 +5860,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="23" spans="1:17" ht="84.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:17" ht="84.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="6" t="s">
         <v>250</v>
       </c>
@@ -5921,7 +5914,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="24" spans="1:17" ht="57.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:17" ht="57.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="6" t="s">
         <v>258</v>
       </c>
@@ -5975,7 +5968,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="25" spans="1:17" ht="71.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:17" ht="71.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="6" t="s">
         <v>269</v>
       </c>
@@ -6299,7 +6292,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="31" spans="1:17" ht="57.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:17" ht="57.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="6" t="s">
         <v>325</v>
       </c>
@@ -6461,7 +6454,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="34" spans="1:17" ht="44.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:17" ht="44.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="6" t="s">
         <v>354</v>
       </c>
@@ -6515,7 +6508,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="35" spans="1:17" ht="57.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:17" ht="57.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="6" t="s">
         <v>363</v>
       </c>
@@ -6569,7 +6562,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="36" spans="1:17" ht="57.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:17" ht="57.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="6" t="s">
         <v>375</v>
       </c>
@@ -6623,7 +6616,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="37" spans="1:17" ht="57.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:17" ht="57.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="6" t="s">
         <v>384</v>
       </c>
@@ -6836,7 +6829,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="41" spans="1:17" ht="44.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:17" ht="44.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="6" t="s">
         <v>424</v>
       </c>
@@ -6890,7 +6883,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="42" spans="1:17" ht="57.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:17" ht="57.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="6" t="s">
         <v>433</v>
       </c>
@@ -6944,7 +6937,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="43" spans="1:17" ht="44.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:17" ht="44.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="6" t="s">
         <v>442</v>
       </c>
@@ -6998,7 +6991,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="44" spans="1:17" ht="57.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:17" ht="57.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="6" t="s">
         <v>453</v>
       </c>
@@ -7214,7 +7207,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="48" spans="1:17" ht="57.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:17" ht="57.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="6" t="s">
         <v>489</v>
       </c>
@@ -7268,7 +7261,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="49" spans="1:17" ht="71.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:17" ht="71.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="6" t="s">
         <v>500</v>
       </c>
@@ -7322,7 +7315,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="50" spans="1:17" ht="71.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:17" ht="71.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="6" t="s">
         <v>510</v>
       </c>
@@ -7427,7 +7420,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="52" spans="1:17" ht="57.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:17" ht="57.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="6" t="s">
         <v>529</v>
       </c>
@@ -7643,7 +7636,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="56" spans="1:17" ht="57.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:17" ht="57.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="6" t="s">
         <v>570</v>
       </c>
@@ -7697,7 +7690,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="57" spans="1:17" ht="44.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:17" ht="44.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="6" t="s">
         <v>579</v>
       </c>
@@ -8237,7 +8230,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="67" spans="1:17" ht="44.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:17" ht="44.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" s="6" t="s">
         <v>671</v>
       </c>
@@ -8450,7 +8443,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="71" spans="1:17" ht="57.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:17" ht="57.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" s="6" t="s">
         <v>709</v>
       </c>
@@ -8525,6 +8518,7 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
@@ -8551,13 +8545,13 @@
       <c r="E1" s="28"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A2" s="31" t="s">
+      <c r="A2" s="30" t="s">
         <v>718</v>
       </c>
-      <c r="B2" s="31"/>
-      <c r="C2" s="31"/>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
     </row>
     <row r="3" spans="1:5" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="15" t="s">
@@ -9969,15 +9963,15 @@
       <c r="G28" s="1"/>
     </row>
     <row r="29" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="29" t="s">
+      <c r="A29" s="31" t="s">
         <v>789</v>
       </c>
-      <c r="B29" s="29"/>
-      <c r="C29" s="29"/>
-      <c r="D29" s="29"/>
-      <c r="E29" s="29"/>
-      <c r="F29" s="29"/>
-      <c r="G29" s="29"/>
+      <c r="B29" s="31"/>
+      <c r="C29" s="31"/>
+      <c r="D29" s="31"/>
+      <c r="E29" s="31"/>
+      <c r="F29" s="31"/>
+      <c r="G29" s="31"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
@@ -10338,16 +10332,16 @@
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{337CDEEC-CE2D-45AB-A77F-FB46EF358718}">
   <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
     <ds:schemaRef ds:uri="8e1efd23-f4ba-42d2-85fd-6a510437bae6"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>